<commit_message>
fix(import): CBO nguồn vốn join dự án trong mẫu import phân khai kinh phí
Hiển thị combo dạng TenNguonVon - TenDuAn, resolve NguonVonId theo junction DuAnNguonVon khi import, đăng ký slug QLDA.Gen và regen template.
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/PrintTemplates/Import_PhanKhaiKinhPhi.xlsx
+++ b/QLDA.WebApi/PrintTemplates/Import_PhanKhaiKinhPhi.xlsx
@@ -1,27 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SER\QLDA.WebApi\PrintTemplates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1CB5B3D-38F1-4E85-9A2C-EDFCE5254B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="2" r:id="rId1"/>
-    <sheet name="ComboData" sheetId="3" r:id="rId2"/>
+    <sheet name="Data" sheetId="2" r:id="rId2"/>
+    <sheet name="ComboData" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
 TRUNG TÂM CHUYỂN ĐỔI SỐ</t>
@@ -35,7 +29,7 @@
     <t>MẪU IMPORT PHÂN KHAI KINH PHÍ</t>
   </si>
   <si>
-    <t>Nhập dữ liệu vào bảng bên dưới. Cột Dự án / Nguồn vốn chọn từ danh sách. Tiền nhập theo đồng.</t>
+    <t>Nhập dữ liệu vào bảng bên dưới. Cột Dự án / Nguồn vốn chọn từ danh sách. Nguồn vốn hiển thị dạng "Tên nguồn vốn - Tên dự án". Tiền nhập theo đồng.</t>
   </si>
   <si>
     <t>Dự án</t>
@@ -65,7 +59,7 @@
     <t>Chọn từ danh sách</t>
   </si>
   <si>
-    <t>Chọn từ danh mục</t>
+    <t>Tên nguồn vốn - Tên dự án</t>
   </si>
   <si>
     <t>Số ≥ 0 (đồng)</t>
@@ -86,12 +80,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="3">
+    <numFmt numFmtId="0" formatCode=""/>
+    <numFmt numFmtId="164" formatCode="#,##0"/>
+    <numFmt numFmtId="165" formatCode="dd/MM/yyyy"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
+      <vertAlign val="baseline"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -99,6 +96,7 @@
     </font>
     <font>
       <b/>
+      <vertAlign val="baseline"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -106,12 +104,14 @@
     </font>
     <font>
       <b/>
+      <vertAlign val="baseline"/>
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="2"/>
     </font>
     <font>
+      <vertAlign val="baseline"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -137,14 +137,24 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+    <border diagonalUp="0" diagonalDown="0">
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal style="none">
+        <color rgb="FF000000"/>
+      </diagonal>
     </border>
-    <border>
+    <border diagonalUp="0" diagonalDown="0">
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -157,88 +167,123 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none">
+        <color rgb="FF000000"/>
+      </diagonal>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
+  <cellStyleXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PhanKhaiKinhPhiImport" displayName="PhanKhaiKinhPhiImport" ref="A5:H7" totalsRowShown="0">
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Dự án"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nguồn vốn"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Kinh phí đề xuất"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Kinh phí phân khai"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Thuyết minh phân khai"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Số tờ trình"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Ngày tờ trình"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Trích yếu"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PhanKhaiKinhPhiImport" displayName="PhanKhaiKinhPhiImport" ref="A5:H7" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Dự án"/>
+    <x:tableColumn id="2" name="Nguồn vốn"/>
+    <x:tableColumn id="3" name="Kinh phí đề xuất"/>
+    <x:tableColumn id="4" name="Kinh phí phân khai"/>
+    <x:tableColumn id="5" name="Thuyết minh phân khai"/>
+    <x:tableColumn id="6" name="Số tờ trình"/>
+    <x:tableColumn id="7" name="Ngày tờ trình"/>
+    <x:tableColumn id="8" name="Trích yếu"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Combo1" displayName="Combo1" ref="A1:A2" totalsRowShown="0">
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="$cbo1"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Combo1" displayName="Combo1" ref="A1:A2" totalsRowShown="0">
+  <x:tableColumns count="1">
+    <x:tableColumn id="1" name="$cbo1"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Combo2" displayName="Combo2" ref="B1:B2" totalsRowShown="0">
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="$cbo2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Combo2" displayName="Combo2" ref="B1:B2" totalsRowShown="0">
+  <x:tableColumns count="1">
+    <x:tableColumn id="1" name="$cbo2"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -525,43 +570,46 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" customWidth="1"/>
-    <col min="2" max="4" width="22.6640625" customWidth="1"/>
-    <col min="5" max="5" width="35.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="35.6640625" customWidth="1"/>
+    <col min="1" max="2" width="40.710625" style="0" customWidth="1"/>
+    <col min="3" max="4" width="22.710625" style="0" customWidth="1"/>
+    <col min="5" max="5" width="35.710625" style="0" customWidth="1"/>
+    <col min="6" max="6" width="18.710625" style="0" customWidth="1"/>
+    <col min="7" max="7" width="16.710625" style="0" customWidth="1"/>
+    <col min="8" max="8" width="35.710625" style="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:8" ht="36" customHeight="1">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="3"/>
+      <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="28" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -573,19 +621,19 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:8" ht="28" customHeight="1">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8">
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
@@ -611,7 +659,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8">
       <c r="A6" s="5" t="s">
         <v>12</v>
       </c>
@@ -637,19 +685,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8">
       <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="6"/>
+      <c r="C7" s="7" t="s"/>
+      <c r="D7" s="7" t="s"/>
+      <c r="E7" s="6" t="s"/>
+      <c r="F7" s="6" t="s"/>
+      <c r="G7" s="8" t="s"/>
+      <c r="H7" s="6" t="s"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -658,31 +706,40 @@
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A4:H4"/>
   </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <headerFooter/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
-  <tableParts count="2">
-    <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
-  </tableParts>
-</worksheet>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:B1"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1" spans="1:2">
+      <x:c r="A1" s="9" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="s">
+        <x:v>18</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="2">
+    <x:tablePart r:id="rId7"/>
+    <x:tablePart r:id="rId8"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>